<commit_message>
Kit Advogados: dados.py como fonte única (casos, propostas, parcelas, caixa, horas); 20 planilhas coerentes entre si (verifica_coerencia: 251 OK), só funções Excel 2007+, valores em cache, NUMEROS.md e telas regeneradas
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146uBo6FVJ2cyEehyP8rK61
</commit_message>
<xml_diff>
--- a/projetos/gestao-ia-planilhas/produto/kit-advogados/03-rotina-da-semana.xlsx
+++ b/projetos/gestao-ia-planilhas/produto/kit-advogados/03-rotina-da-semana.xlsx
@@ -825,7 +825,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>O escritório fictício registrou de 20/07 a 07/09/2026 (S29 a S36). O Painel sempre olha as últimas semanas registradas, então o exemplo continua fazendo sentido em qualquer data.</t>
+          <t>O escritório fictício registrou de 20/07 a 07/09/2026 (S29 a S36). O Painel sempre olha as últimas semanas registradas, então o exemplo continua fazendo sentido em qualquer data. Em janeiro de 2027, troque a segunda-feira da semana 1 em Config (veja a nota lá).</t>
         </is>
       </c>
     </row>
@@ -873,7 +873,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Excel 2019 ou mais novo, Microsoft 365 ou Google Sheets. No celular abre nos aplicativos; para preencher, use o computador.</t>
+          <t>Excel 2016 ou mais novo, Microsoft 365 ou Google Sheets (só funções do Excel 2007+; nada de MÍNIMOSES, MÁXIMOSES ou UNIRTEXTO). No celular abre nos aplicativos; para preencher, use o computador.</t>
         </is>
       </c>
     </row>
@@ -942,9 +942,9 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="5">
+      <c r="A1" s="5" t="str">
         <f>Config!$B$4&amp;" · Aderência à rotina · "&amp;TEXT(Config!$B$5,"dd/mm/yyyy")</f>
-        <v/>
+        <v>Ferraz &amp; Lima Advocacia (exemplo fictício) · Aderência à rotina · 14/09/2026</v>
       </c>
     </row>
     <row r="2">
@@ -985,29 +985,29 @@
         </is>
       </c>
       <c r="K4" s="14">
-        <f>IFERROR(_xlfn.MAXIFS(Rotina!$E$2:$BD$2,Rotina!$E$31:$BD$31,"&gt;0"),0)</f>
-        <v/>
+        <f>SUMPRODUCT(MAX((Rotina!$E$31:$BD$31&gt;0)*Rotina!$E$2:$BD$2))</f>
+        <v>36</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="15">
         <f>IF(OR($K$4=0,$K$7=0),"",SUMPRODUCT((Rotina!$E$2:$BD$2&gt;=$K$4-3)*(Rotina!$E$2:$BD$2&lt;=$K$4)*Rotina!$E$30:$BD$30)/($K$6*$K$7))</f>
-        <v/>
+        <v>0.833333333333333</v>
       </c>
       <c r="B5" s="8" t="n"/>
-      <c r="C5" s="16">
+      <c r="C5" s="16" t="str">
         <f>"S"&amp;$K$5&amp;" · "&amp;TEXT(Config!$B$6+7*($K$5-1),"dd/mm")</f>
-        <v/>
+        <v>S37 · 14/09</v>
       </c>
       <c r="D5" s="10" t="n"/>
-      <c r="E5" s="17">
+      <c r="E5" s="17" t="str">
         <f>IF($K$4=0,"nenhuma","S"&amp;$K$4&amp;" · "&amp;TEXT(Config!$B$6+7*($K$4-1),"dd/mm"))</f>
-        <v/>
+        <v>S36 · 07/09</v>
       </c>
       <c r="F5" s="8" t="n"/>
       <c r="G5" s="18">
         <f>SUM(Rotina!$C$5:$C$28)</f>
-        <v/>
+        <v>30</v>
       </c>
       <c r="H5" s="12" t="n"/>
       <c r="J5" s="13" t="inlineStr">
@@ -1017,7 +1017,7 @@
       </c>
       <c r="K5" s="14">
         <f>MIN(52,MAX(1,INT((Config!$B$5-Config!$B$6)/7)+1))</f>
-        <v/>
+        <v>37</v>
       </c>
     </row>
     <row r="6">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="K6" s="14">
         <f>MIN(4,K4)</f>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="K7" s="14">
         <f>COUNTA(Rotina!$B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
     </row>
     <row r="8" ht="26" customHeight="1">
@@ -1087,23 +1087,23 @@
       </c>
       <c r="B9" s="22">
         <f>COUNTIFS(Rotina!$A$5:$A$28,A9,Rotina!$B$5:$B$28,"&lt;&gt;")</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="C9" s="22">
         <f>SUMIFS(Rotina!$C$5:$C$28,Rotina!$A$5:$A$28,A9,Rotina!$B$5:$B$28,"&lt;&gt;")</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="D9" s="22">
         <f>IF($K$4=0,"",SUMIFS($E$29:$E$52,$A$29:$A$52,A9))</f>
-        <v/>
+        <v>15</v>
       </c>
       <c r="E9" s="22">
         <f>IF($K$4=0,"",B9*$K$6)</f>
-        <v/>
+        <v>16</v>
       </c>
       <c r="F9" s="23">
         <f>IF(OR(E9="",E9=0),"",D9/E9)</f>
-        <v/>
+        <v>0.9375</v>
       </c>
     </row>
     <row r="10">
@@ -1114,19 +1114,19 @@
       </c>
       <c r="B10" s="22">
         <f>COUNTIFS(Rotina!$A$5:$A$28,A10,Rotina!$B$5:$B$28,"&lt;&gt;")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C10" s="22">
         <f>SUMIFS(Rotina!$C$5:$C$28,Rotina!$A$5:$A$28,A10,Rotina!$B$5:$B$28,"&lt;&gt;")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D10" s="22">
         <f>IF($K$4=0,"",SUMIFS($E$29:$E$52,$A$29:$A$52,A10))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E10" s="22">
         <f>IF($K$4=0,"",B10*$K$6)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F10" s="23">
         <f>IF(OR(E10="",E10=0),"",D10/E10)</f>
@@ -1141,19 +1141,19 @@
       </c>
       <c r="B11" s="22">
         <f>COUNTIFS(Rotina!$A$5:$A$28,A11,Rotina!$B$5:$B$28,"&lt;&gt;")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C11" s="22">
         <f>SUMIFS(Rotina!$C$5:$C$28,Rotina!$A$5:$A$28,A11,Rotina!$B$5:$B$28,"&lt;&gt;")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D11" s="22">
         <f>IF($K$4=0,"",SUMIFS($E$29:$E$52,$A$29:$A$52,A11))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E11" s="22">
         <f>IF($K$4=0,"",B11*$K$6)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F11" s="23">
         <f>IF(OR(E11="",E11=0),"",D11/E11)</f>
@@ -1168,19 +1168,19 @@
       </c>
       <c r="B12" s="22">
         <f>COUNTIFS(Rotina!$A$5:$A$28,A12,Rotina!$B$5:$B$28,"&lt;&gt;")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C12" s="22">
         <f>SUMIFS(Rotina!$C$5:$C$28,Rotina!$A$5:$A$28,A12,Rotina!$B$5:$B$28,"&lt;&gt;")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D12" s="22">
         <f>IF($K$4=0,"",SUMIFS($E$29:$E$52,$A$29:$A$52,A12))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E12" s="22">
         <f>IF($K$4=0,"",B12*$K$6)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F12" s="23">
         <f>IF(OR(E12="",E12=0),"",D12/E12)</f>
@@ -1195,23 +1195,23 @@
       </c>
       <c r="B13" s="22">
         <f>COUNTIFS(Rotina!$A$5:$A$28,A13,Rotina!$B$5:$B$28,"&lt;&gt;")</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="C13" s="22">
         <f>SUMIFS(Rotina!$C$5:$C$28,Rotina!$A$5:$A$28,A13,Rotina!$B$5:$B$28,"&lt;&gt;")</f>
-        <v/>
+        <v>18</v>
       </c>
       <c r="D13" s="22">
         <f>IF($K$4=0,"",SUMIFS($E$29:$E$52,$A$29:$A$52,A13))</f>
-        <v/>
+        <v>15</v>
       </c>
       <c r="E13" s="22">
         <f>IF($K$4=0,"",B13*$K$6)</f>
-        <v/>
+        <v>20</v>
       </c>
       <c r="F13" s="23">
         <f>IF(OR(E13="",E13=0),"",D13/E13)</f>
-        <v/>
+        <v>0.75</v>
       </c>
     </row>
     <row r="15">
@@ -1259,250 +1259,250 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="22">
+      <c r="A17" s="22" t="str">
         <f>IF(($K$4-7)&lt;1,"","S"&amp;($K$4-7))</f>
-        <v/>
+        <v>S29</v>
       </c>
       <c r="B17" s="24">
         <f>IF(A17="","",INDEX(Rotina!$E$3:$BD$3,($K$4-7)))</f>
-        <v/>
+        <v>46223.0</v>
       </c>
       <c r="C17" s="22">
         <f>IF(A17="","",INDEX(Rotina!$E$30:$BD$30,($K$4-7)))</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="D17" s="22">
         <f>IF(A17="","",INDEX(Rotina!$E$32:$BD$32,($K$4-7)))</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="E17" s="23">
         <f>IF(OR(A17="",D17=0),"",C17/D17)</f>
-        <v/>
+        <v>0.666666666666667</v>
       </c>
       <c r="F17" s="22">
         <f>IF(A17="","",INDEX(Rotina!$E$34:$BD$34,($K$4-7)))</f>
-        <v/>
-      </c>
-      <c r="G17" s="25">
+        <v>19</v>
+      </c>
+      <c r="G17" s="25" t="str">
         <f>IF(E17="","",REPT("█",ROUND(E17*10,0)))</f>
-        <v/>
+        <v>███████</v>
       </c>
       <c r="H17" s="26" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="22">
+      <c r="A18" s="22" t="str">
         <f>IF(($K$4-6)&lt;1,"","S"&amp;($K$4-6))</f>
-        <v/>
+        <v>S30</v>
       </c>
       <c r="B18" s="24">
         <f>IF(A18="","",INDEX(Rotina!$E$3:$BD$3,($K$4-6)))</f>
-        <v/>
+        <v>46230.0</v>
       </c>
       <c r="C18" s="22">
         <f>IF(A18="","",INDEX(Rotina!$E$30:$BD$30,($K$4-6)))</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="D18" s="22">
         <f>IF(A18="","",INDEX(Rotina!$E$32:$BD$32,($K$4-6)))</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="E18" s="23">
         <f>IF(OR(A18="",D18=0),"",C18/D18)</f>
-        <v/>
+        <v>0.777777777777778</v>
       </c>
       <c r="F18" s="22">
         <f>IF(A18="","",INDEX(Rotina!$E$34:$BD$34,($K$4-6)))</f>
-        <v/>
-      </c>
-      <c r="G18" s="25">
+        <v>24</v>
+      </c>
+      <c r="G18" s="25" t="str">
         <f>IF(E18="","",REPT("█",ROUND(E18*10,0)))</f>
-        <v/>
+        <v>████████</v>
       </c>
       <c r="H18" s="26" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="22">
+      <c r="A19" s="22" t="str">
         <f>IF(($K$4-5)&lt;1,"","S"&amp;($K$4-5))</f>
-        <v/>
+        <v>S31</v>
       </c>
       <c r="B19" s="24">
         <f>IF(A19="","",INDEX(Rotina!$E$3:$BD$3,($K$4-5)))</f>
-        <v/>
+        <v>46237.0</v>
       </c>
       <c r="C19" s="22">
         <f>IF(A19="","",INDEX(Rotina!$E$30:$BD$30,($K$4-5)))</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="D19" s="22">
         <f>IF(A19="","",INDEX(Rotina!$E$32:$BD$32,($K$4-5)))</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="E19" s="23">
         <f>IF(OR(A19="",D19=0),"",C19/D19)</f>
-        <v/>
+        <v>0.888888888888889</v>
       </c>
       <c r="F19" s="22">
         <f>IF(A19="","",INDEX(Rotina!$E$34:$BD$34,($K$4-5)))</f>
-        <v/>
-      </c>
-      <c r="G19" s="25">
+        <v>27</v>
+      </c>
+      <c r="G19" s="25" t="str">
         <f>IF(E19="","",REPT("█",ROUND(E19*10,0)))</f>
-        <v/>
+        <v>█████████</v>
       </c>
       <c r="H19" s="26" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="22">
+      <c r="A20" s="22" t="str">
         <f>IF(($K$4-4)&lt;1,"","S"&amp;($K$4-4))</f>
-        <v/>
+        <v>S32</v>
       </c>
       <c r="B20" s="24">
         <f>IF(A20="","",INDEX(Rotina!$E$3:$BD$3,($K$4-4)))</f>
-        <v/>
+        <v>46244.0</v>
       </c>
       <c r="C20" s="22">
         <f>IF(A20="","",INDEX(Rotina!$E$30:$BD$30,($K$4-4)))</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="D20" s="22">
         <f>IF(A20="","",INDEX(Rotina!$E$32:$BD$32,($K$4-4)))</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="E20" s="23">
         <f>IF(OR(A20="",D20=0),"",C20/D20)</f>
-        <v/>
+        <v>0.888888888888889</v>
       </c>
       <c r="F20" s="22">
         <f>IF(A20="","",INDEX(Rotina!$E$34:$BD$34,($K$4-4)))</f>
-        <v/>
-      </c>
-      <c r="G20" s="25">
+        <v>27</v>
+      </c>
+      <c r="G20" s="25" t="str">
         <f>IF(E20="","",REPT("█",ROUND(E20*10,0)))</f>
-        <v/>
+        <v>█████████</v>
       </c>
       <c r="H20" s="26" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="22">
+      <c r="A21" s="22" t="str">
         <f>IF(($K$4-3)&lt;1,"","S"&amp;($K$4-3))</f>
-        <v/>
+        <v>S33</v>
       </c>
       <c r="B21" s="24">
         <f>IF(A21="","",INDEX(Rotina!$E$3:$BD$3,($K$4-3)))</f>
-        <v/>
+        <v>46251.0</v>
       </c>
       <c r="C21" s="22">
         <f>IF(A21="","",INDEX(Rotina!$E$30:$BD$30,($K$4-3)))</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="D21" s="22">
         <f>IF(A21="","",INDEX(Rotina!$E$32:$BD$32,($K$4-3)))</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="E21" s="23">
         <f>IF(OR(A21="",D21=0),"",C21/D21)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="F21" s="22">
         <f>IF(A21="","",INDEX(Rotina!$E$34:$BD$34,($K$4-3)))</f>
-        <v/>
-      </c>
-      <c r="G21" s="25">
+        <v>30</v>
+      </c>
+      <c r="G21" s="25" t="str">
         <f>IF(E21="","",REPT("█",ROUND(E21*10,0)))</f>
-        <v/>
+        <v>██████████</v>
       </c>
       <c r="H21" s="26" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="22">
+      <c r="A22" s="22" t="str">
         <f>IF(($K$4-2)&lt;1,"","S"&amp;($K$4-2))</f>
-        <v/>
+        <v>S34</v>
       </c>
       <c r="B22" s="24">
         <f>IF(A22="","",INDEX(Rotina!$E$3:$BD$3,($K$4-2)))</f>
-        <v/>
+        <v>46258.0</v>
       </c>
       <c r="C22" s="22">
         <f>IF(A22="","",INDEX(Rotina!$E$30:$BD$30,($K$4-2)))</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="D22" s="22">
         <f>IF(A22="","",INDEX(Rotina!$E$32:$BD$32,($K$4-2)))</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="E22" s="23">
         <f>IF(OR(A22="",D22=0),"",C22/D22)</f>
-        <v/>
+        <v>0.777777777777778</v>
       </c>
       <c r="F22" s="22">
         <f>IF(A22="","",INDEX(Rotina!$E$34:$BD$34,($K$4-2)))</f>
-        <v/>
-      </c>
-      <c r="G22" s="25">
+        <v>23</v>
+      </c>
+      <c r="G22" s="25" t="str">
         <f>IF(E22="","",REPT("█",ROUND(E22*10,0)))</f>
-        <v/>
+        <v>████████</v>
       </c>
       <c r="H22" s="26" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="22">
+      <c r="A23" s="22" t="str">
         <f>IF(($K$4-1)&lt;1,"","S"&amp;($K$4-1))</f>
-        <v/>
+        <v>S35</v>
       </c>
       <c r="B23" s="24">
         <f>IF(A23="","",INDEX(Rotina!$E$3:$BD$3,($K$4-1)))</f>
-        <v/>
+        <v>46265.0</v>
       </c>
       <c r="C23" s="22">
         <f>IF(A23="","",INDEX(Rotina!$E$30:$BD$30,($K$4-1)))</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="D23" s="22">
         <f>IF(A23="","",INDEX(Rotina!$E$32:$BD$32,($K$4-1)))</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="E23" s="23">
         <f>IF(OR(A23="",D23=0),"",C23/D23)</f>
-        <v/>
+        <v>0.777777777777778</v>
       </c>
       <c r="F23" s="22">
         <f>IF(A23="","",INDEX(Rotina!$E$34:$BD$34,($K$4-1)))</f>
-        <v/>
-      </c>
-      <c r="G23" s="25">
+        <v>24</v>
+      </c>
+      <c r="G23" s="25" t="str">
         <f>IF(E23="","",REPT("█",ROUND(E23*10,0)))</f>
-        <v/>
+        <v>████████</v>
       </c>
       <c r="H23" s="26" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="22">
+      <c r="A24" s="22" t="str">
         <f>IF(($K$4-0)&lt;1,"","S"&amp;($K$4-0))</f>
-        <v/>
+        <v>S36</v>
       </c>
       <c r="B24" s="24">
         <f>IF(A24="","",INDEX(Rotina!$E$3:$BD$3,($K$4-0)))</f>
-        <v/>
+        <v>46272.0</v>
       </c>
       <c r="C24" s="22">
         <f>IF(A24="","",INDEX(Rotina!$E$30:$BD$30,($K$4-0)))</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="D24" s="22">
         <f>IF(A24="","",INDEX(Rotina!$E$32:$BD$32,($K$4-0)))</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="E24" s="23">
         <f>IF(OR(A24="",D24=0),"",C24/D24)</f>
-        <v/>
+        <v>0.777777777777778</v>
       </c>
       <c r="F24" s="22">
         <f>IF(A24="","",INDEX(Rotina!$E$34:$BD$34,($K$4-0)))</f>
-        <v/>
-      </c>
-      <c r="G24" s="25">
+        <v>25</v>
+      </c>
+      <c r="G24" s="25" t="str">
         <f>IF(E24="","",REPT("█",ROUND(E24*10,0)))</f>
-        <v/>
+        <v>████████</v>
       </c>
       <c r="H24" s="26" t="n"/>
     </row>
@@ -1563,33 +1563,33 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="22">
+      <c r="A29" s="22" t="str">
         <f>IF(Rotina!$B5="","",Rotina!$A5)</f>
-        <v/>
-      </c>
-      <c r="B29" s="21">
+        <v>Segunda</v>
+      </c>
+      <c r="B29" s="21" t="str">
         <f>IF(Rotina!$B5="","",Rotina!$B5)</f>
-        <v/>
+        <v>Abrir a Agenda de prazos: resolver ou reagendar os atrasados</v>
       </c>
       <c r="C29" s="22">
         <f>IF(Rotina!$B5="","",Rotina!$C5)</f>
-        <v/>
-      </c>
-      <c r="D29" s="22">
+        <v>4</v>
+      </c>
+      <c r="D29" s="22" t="str">
         <f>IF(Rotina!$B5="","",Rotina!$D5)</f>
-        <v/>
+        <v>Marina Ferraz</v>
       </c>
       <c r="E29" s="22">
         <f>IF(OR(Rotina!$B5="",$K$4=0),"",SUMPRODUCT((Rotina!$E$5:$BD$5="Sim")*(Rotina!$E$2:$BD$2&gt;=$K$4-3)*(Rotina!$E$2:$BD$2&lt;=$K$4)))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="F29" s="22">
         <f>IF(E29="","",$K$6)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="G29" s="23">
         <f>IF(OR(E29="",F29=0),"",E29/F29)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="H29" s="21">
         <f>IF(G29="","",IF(G29&lt;0.5,"Pulada na maioria das semanas",IF(G29&lt;0.75,"Pulada às vezes","")))</f>
@@ -1597,33 +1597,33 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="22">
+      <c r="A30" s="22" t="str">
         <f>IF(Rotina!$B6="","",Rotina!$A6)</f>
-        <v/>
-      </c>
-      <c r="B30" s="21">
+        <v>Segunda</v>
+      </c>
+      <c r="B30" s="21" t="str">
         <f>IF(Rotina!$B6="","",Rotina!$B6)</f>
-        <v/>
+        <v>Confirmar com cada responsável os prazos dos próximos 7 dias</v>
       </c>
       <c r="C30" s="22">
         <f>IF(Rotina!$B6="","",Rotina!$C6)</f>
-        <v/>
-      </c>
-      <c r="D30" s="22">
+        <v>3</v>
+      </c>
+      <c r="D30" s="22" t="str">
         <f>IF(Rotina!$B6="","",Rotina!$D6)</f>
-        <v/>
+        <v>Rafael Lima</v>
       </c>
       <c r="E30" s="22">
         <f>IF(OR(Rotina!$B6="",$K$4=0),"",SUMPRODUCT((Rotina!$E$6:$BD$6="Sim")*(Rotina!$E$2:$BD$2&gt;=$K$4-3)*(Rotina!$E$2:$BD$2&lt;=$K$4)))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="F30" s="22">
         <f>IF(E30="","",$K$6)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="G30" s="23">
         <f>IF(OR(E30="",F30=0),"",E30/F30)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="H30" s="21">
         <f>IF(G30="","",IF(G30&lt;0.5,"Pulada na maioria das semanas",IF(G30&lt;0.75,"Pulada às vezes","")))</f>
@@ -1631,33 +1631,33 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="22">
+      <c r="A31" s="22" t="str">
         <f>IF(Rotina!$B7="","",Rotina!$A7)</f>
-        <v/>
-      </c>
-      <c r="B31" s="21">
+        <v>Segunda</v>
+      </c>
+      <c r="B31" s="21" t="str">
         <f>IF(Rotina!$B7="","",Rotina!$B7)</f>
-        <v/>
+        <v>Registrar os prazos e audiências novos que chegaram</v>
       </c>
       <c r="C31" s="22">
         <f>IF(Rotina!$B7="","",Rotina!$C7)</f>
-        <v/>
-      </c>
-      <c r="D31" s="22">
+        <v>3</v>
+      </c>
+      <c r="D31" s="22" t="str">
         <f>IF(Rotina!$B7="","",Rotina!$D7)</f>
-        <v/>
+        <v>Júlia Prado</v>
       </c>
       <c r="E31" s="22">
         <f>IF(OR(Rotina!$B7="",$K$4=0),"",SUMPRODUCT((Rotina!$E$7:$BD$7="Sim")*(Rotina!$E$2:$BD$2&gt;=$K$4-3)*(Rotina!$E$2:$BD$2&lt;=$K$4)))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="F31" s="22">
         <f>IF(E31="","",$K$6)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="G31" s="23">
         <f>IF(OR(E31="",F31=0),"",E31/F31)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="H31" s="21">
         <f>IF(G31="","",IF(G31&lt;0.5,"Pulada na maioria das semanas",IF(G31&lt;0.75,"Pulada às vezes","")))</f>
@@ -1665,33 +1665,33 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="22">
+      <c r="A32" s="22" t="str">
         <f>IF(Rotina!$B8="","",Rotina!$A8)</f>
-        <v/>
-      </c>
-      <c r="B32" s="21">
+        <v>Segunda</v>
+      </c>
+      <c r="B32" s="21" t="str">
         <f>IF(Rotina!$B8="","",Rotina!$B8)</f>
-        <v/>
+        <v>Atualizar fase e próxima ação dos casos movimentados</v>
       </c>
       <c r="C32" s="22">
         <f>IF(Rotina!$B8="","",Rotina!$C8)</f>
-        <v/>
-      </c>
-      <c r="D32" s="22">
+        <v>2</v>
+      </c>
+      <c r="D32" s="22" t="str">
         <f>IF(Rotina!$B8="","",Rotina!$D8)</f>
-        <v/>
+        <v>Júlia Prado</v>
       </c>
       <c r="E32" s="22">
         <f>IF(OR(Rotina!$B8="",$K$4=0),"",SUMPRODUCT((Rotina!$E$8:$BD$8="Sim")*(Rotina!$E$2:$BD$2&gt;=$K$4-3)*(Rotina!$E$2:$BD$2&lt;=$K$4)))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="F32" s="22">
         <f>IF(E32="","",$K$6)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="G32" s="23">
         <f>IF(OR(E32="",F32=0),"",E32/F32)</f>
-        <v/>
+        <v>0.75</v>
       </c>
       <c r="H32" s="21">
         <f>IF(G32="","",IF(G32&lt;0.5,"Pulada na maioria das semanas",IF(G32&lt;0.75,"Pulada às vezes","")))</f>
@@ -1699,33 +1699,33 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="22">
+      <c r="A33" s="22" t="str">
         <f>IF(Rotina!$B9="","",Rotina!$A9)</f>
-        <v/>
-      </c>
-      <c r="B33" s="21">
+        <v>Sexta</v>
+      </c>
+      <c r="B33" s="21" t="str">
         <f>IF(Rotina!$B9="","",Rotina!$B9)</f>
-        <v/>
+        <v>Lançar as entradas e saídas da semana no caixa</v>
       </c>
       <c r="C33" s="22">
         <f>IF(Rotina!$B9="","",Rotina!$C9)</f>
-        <v/>
-      </c>
-      <c r="D33" s="22">
+        <v>5</v>
+      </c>
+      <c r="D33" s="22" t="str">
         <f>IF(Rotina!$B9="","",Rotina!$D9)</f>
-        <v/>
+        <v>Marina Ferraz</v>
       </c>
       <c r="E33" s="22">
         <f>IF(OR(Rotina!$B9="",$K$4=0),"",SUMPRODUCT((Rotina!$E$9:$BD$9="Sim")*(Rotina!$E$2:$BD$2&gt;=$K$4-3)*(Rotina!$E$2:$BD$2&lt;=$K$4)))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="F33" s="22">
         <f>IF(E33="","",$K$6)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="G33" s="23">
         <f>IF(OR(E33="",F33=0),"",E33/F33)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="H33" s="21">
         <f>IF(G33="","",IF(G33&lt;0.5,"Pulada na maioria das semanas",IF(G33&lt;0.75,"Pulada às vezes","")))</f>
@@ -1733,33 +1733,33 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="22">
+      <c r="A34" s="22" t="str">
         <f>IF(Rotina!$B10="","",Rotina!$A10)</f>
-        <v/>
-      </c>
-      <c r="B34" s="21">
+        <v>Sexta</v>
+      </c>
+      <c r="B34" s="21" t="str">
         <f>IF(Rotina!$B10="","",Rotina!$B10)</f>
-        <v/>
+        <v>Marcar as parcelas recebidas e as atrasadas</v>
       </c>
       <c r="C34" s="22">
         <f>IF(Rotina!$B10="","",Rotina!$C10)</f>
-        <v/>
-      </c>
-      <c r="D34" s="22">
+        <v>3</v>
+      </c>
+      <c r="D34" s="22" t="str">
         <f>IF(Rotina!$B10="","",Rotina!$D10)</f>
-        <v/>
+        <v>Marina Ferraz</v>
       </c>
       <c r="E34" s="22">
         <f>IF(OR(Rotina!$B10="",$K$4=0),"",SUMPRODUCT((Rotina!$E$10:$BD$10="Sim")*(Rotina!$E$2:$BD$2&gt;=$K$4-3)*(Rotina!$E$2:$BD$2&lt;=$K$4)))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="F34" s="22">
         <f>IF(E34="","",$K$6)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="G34" s="23">
         <f>IF(OR(E34="",F34=0),"",E34/F34)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="H34" s="21">
         <f>IF(G34="","",IF(G34&lt;0.5,"Pulada na maioria das semanas",IF(G34&lt;0.75,"Pulada às vezes","")))</f>
@@ -1767,33 +1767,33 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="22">
+      <c r="A35" s="22" t="str">
         <f>IF(Rotina!$B11="","",Rotina!$A11)</f>
-        <v/>
-      </c>
-      <c r="B35" s="21">
+        <v>Sexta</v>
+      </c>
+      <c r="B35" s="21" t="str">
         <f>IF(Rotina!$B11="","",Rotina!$B11)</f>
-        <v/>
+        <v>Registrar as horas da semana por caso</v>
       </c>
       <c r="C35" s="22">
         <f>IF(Rotina!$B11="","",Rotina!$C11)</f>
-        <v/>
-      </c>
-      <c r="D35" s="22">
+        <v>4</v>
+      </c>
+      <c r="D35" s="22" t="str">
         <f>IF(Rotina!$B11="","",Rotina!$D11)</f>
-        <v/>
+        <v>Rafael Lima</v>
       </c>
       <c r="E35" s="22">
         <f>IF(OR(Rotina!$B11="",$K$4=0),"",SUMPRODUCT((Rotina!$E$11:$BD$11="Sim")*(Rotina!$E$2:$BD$2&gt;=$K$4-3)*(Rotina!$E$2:$BD$2&lt;=$K$4)))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="F35" s="22">
         <f>IF(E35="","",$K$6)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="G35" s="23">
         <f>IF(OR(E35="",F35=0),"",E35/F35)</f>
-        <v/>
+        <v>0.75</v>
       </c>
       <c r="H35" s="21">
         <f>IF(G35="","",IF(G35&lt;0.5,"Pulada na maioria das semanas",IF(G35&lt;0.75,"Pulada às vezes","")))</f>
@@ -1801,67 +1801,67 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="22">
+      <c r="A36" s="22" t="str">
         <f>IF(Rotina!$B12="","",Rotina!$A12)</f>
-        <v/>
-      </c>
-      <c r="B36" s="21">
+        <v>Sexta</v>
+      </c>
+      <c r="B36" s="21" t="str">
         <f>IF(Rotina!$B12="","",Rotina!$B12)</f>
-        <v/>
+        <v>Enviar a cobrança educada das parcelas atrasadas</v>
       </c>
       <c r="C36" s="22">
         <f>IF(Rotina!$B12="","",Rotina!$C12)</f>
-        <v/>
-      </c>
-      <c r="D36" s="22">
+        <v>3</v>
+      </c>
+      <c r="D36" s="22" t="str">
         <f>IF(Rotina!$B12="","",Rotina!$D12)</f>
-        <v/>
+        <v>Rafael Lima</v>
       </c>
       <c r="E36" s="22">
         <f>IF(OR(Rotina!$B12="",$K$4=0),"",SUMPRODUCT((Rotina!$E$12:$BD$12="Sim")*(Rotina!$E$2:$BD$2&gt;=$K$4-3)*(Rotina!$E$2:$BD$2&lt;=$K$4)))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="F36" s="22">
         <f>IF(E36="","",$K$6)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="G36" s="23">
         <f>IF(OR(E36="",F36=0),"",E36/F36)</f>
-        <v/>
-      </c>
-      <c r="H36" s="21">
+        <v>0.25</v>
+      </c>
+      <c r="H36" s="21" t="str">
         <f>IF(G36="","",IF(G36&lt;0.5,"Pulada na maioria das semanas",IF(G36&lt;0.75,"Pulada às vezes","")))</f>
-        <v/>
+        <v>Pulada na maioria das semanas</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="22">
+      <c r="A37" s="22" t="str">
         <f>IF(Rotina!$B13="","",Rotina!$A13)</f>
-        <v/>
-      </c>
-      <c r="B37" s="21">
+        <v>Sexta</v>
+      </c>
+      <c r="B37" s="21" t="str">
         <f>IF(Rotina!$B13="","",Rotina!$B13)</f>
-        <v/>
+        <v>Olhar o painel do escritório e anotar até 3 decisões</v>
       </c>
       <c r="C37" s="22">
         <f>IF(Rotina!$B13="","",Rotina!$C13)</f>
-        <v/>
-      </c>
-      <c r="D37" s="22">
+        <v>3</v>
+      </c>
+      <c r="D37" s="22" t="str">
         <f>IF(Rotina!$B13="","",Rotina!$D13)</f>
-        <v/>
+        <v>Marina Ferraz</v>
       </c>
       <c r="E37" s="22">
         <f>IF(OR(Rotina!$B13="",$K$4=0),"",SUMPRODUCT((Rotina!$E$13:$BD$13="Sim")*(Rotina!$E$2:$BD$2&gt;=$K$4-3)*(Rotina!$E$2:$BD$2&lt;=$K$4)))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="F37" s="22">
         <f>IF(E37="","",$K$6)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="G37" s="23">
         <f>IF(OR(E37="",F37=0),"",E37/F37)</f>
-        <v/>
+        <v>0.75</v>
       </c>
       <c r="H37" s="21">
         <f>IF(G37="","",IF(G37&lt;0.5,"Pulada na maioria das semanas",IF(G37&lt;0.75,"Pulada às vezes","")))</f>
@@ -2478,7 +2478,7 @@
       </c>
       <c r="B5" s="29">
         <f>TODAY()</f>
-        <v/>
+        <v>46279.0</v>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
@@ -2498,6 +2498,13 @@
       <c r="C6" s="13" t="inlineStr">
         <is>
           <t>Sugestão: a primeira segunda-feira do ano. As 52 colunas da aba Rotina contam a partir daqui. O exemplo está preenchido de 20/07 a 07/09/2026 (S29 a S36).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Virada do ano: em janeiro de 2027, salve uma cópia desta planilha, troque a data acima pela primeira segunda-feira de 2027 (04/01/2027) e limpe as marcações da aba Rotina. As 52 semanas recomeçam.</t>
         </is>
       </c>
     </row>
@@ -2812,211 +2819,211 @@
       </c>
       <c r="E3" s="32">
         <f>Config!$B$6+0</f>
-        <v/>
+        <v>46027.0</v>
       </c>
       <c r="F3" s="32">
         <f>Config!$B$6+7</f>
-        <v/>
+        <v>46034.0</v>
       </c>
       <c r="G3" s="32">
         <f>Config!$B$6+14</f>
-        <v/>
+        <v>46041.0</v>
       </c>
       <c r="H3" s="32">
         <f>Config!$B$6+21</f>
-        <v/>
+        <v>46048.0</v>
       </c>
       <c r="I3" s="32">
         <f>Config!$B$6+28</f>
-        <v/>
+        <v>46055.0</v>
       </c>
       <c r="J3" s="32">
         <f>Config!$B$6+35</f>
-        <v/>
+        <v>46062.0</v>
       </c>
       <c r="K3" s="32">
         <f>Config!$B$6+42</f>
-        <v/>
+        <v>46069.0</v>
       </c>
       <c r="L3" s="32">
         <f>Config!$B$6+49</f>
-        <v/>
+        <v>46076.0</v>
       </c>
       <c r="M3" s="32">
         <f>Config!$B$6+56</f>
-        <v/>
+        <v>46083.0</v>
       </c>
       <c r="N3" s="32">
         <f>Config!$B$6+63</f>
-        <v/>
+        <v>46090.0</v>
       </c>
       <c r="O3" s="32">
         <f>Config!$B$6+70</f>
-        <v/>
+        <v>46097.0</v>
       </c>
       <c r="P3" s="32">
         <f>Config!$B$6+77</f>
-        <v/>
+        <v>46104.0</v>
       </c>
       <c r="Q3" s="32">
         <f>Config!$B$6+84</f>
-        <v/>
+        <v>46111.0</v>
       </c>
       <c r="R3" s="32">
         <f>Config!$B$6+91</f>
-        <v/>
+        <v>46118.0</v>
       </c>
       <c r="S3" s="32">
         <f>Config!$B$6+98</f>
-        <v/>
+        <v>46125.0</v>
       </c>
       <c r="T3" s="32">
         <f>Config!$B$6+105</f>
-        <v/>
+        <v>46132.0</v>
       </c>
       <c r="U3" s="32">
         <f>Config!$B$6+112</f>
-        <v/>
+        <v>46139.0</v>
       </c>
       <c r="V3" s="32">
         <f>Config!$B$6+119</f>
-        <v/>
+        <v>46146.0</v>
       </c>
       <c r="W3" s="32">
         <f>Config!$B$6+126</f>
-        <v/>
+        <v>46153.0</v>
       </c>
       <c r="X3" s="32">
         <f>Config!$B$6+133</f>
-        <v/>
+        <v>46160.0</v>
       </c>
       <c r="Y3" s="32">
         <f>Config!$B$6+140</f>
-        <v/>
+        <v>46167.0</v>
       </c>
       <c r="Z3" s="32">
         <f>Config!$B$6+147</f>
-        <v/>
+        <v>46174.0</v>
       </c>
       <c r="AA3" s="32">
         <f>Config!$B$6+154</f>
-        <v/>
+        <v>46181.0</v>
       </c>
       <c r="AB3" s="32">
         <f>Config!$B$6+161</f>
-        <v/>
+        <v>46188.0</v>
       </c>
       <c r="AC3" s="32">
         <f>Config!$B$6+168</f>
-        <v/>
+        <v>46195.0</v>
       </c>
       <c r="AD3" s="32">
         <f>Config!$B$6+175</f>
-        <v/>
+        <v>46202.0</v>
       </c>
       <c r="AE3" s="32">
         <f>Config!$B$6+182</f>
-        <v/>
+        <v>46209.0</v>
       </c>
       <c r="AF3" s="32">
         <f>Config!$B$6+189</f>
-        <v/>
+        <v>46216.0</v>
       </c>
       <c r="AG3" s="32">
         <f>Config!$B$6+196</f>
-        <v/>
+        <v>46223.0</v>
       </c>
       <c r="AH3" s="32">
         <f>Config!$B$6+203</f>
-        <v/>
+        <v>46230.0</v>
       </c>
       <c r="AI3" s="32">
         <f>Config!$B$6+210</f>
-        <v/>
+        <v>46237.0</v>
       </c>
       <c r="AJ3" s="32">
         <f>Config!$B$6+217</f>
-        <v/>
+        <v>46244.0</v>
       </c>
       <c r="AK3" s="32">
         <f>Config!$B$6+224</f>
-        <v/>
+        <v>46251.0</v>
       </c>
       <c r="AL3" s="32">
         <f>Config!$B$6+231</f>
-        <v/>
+        <v>46258.0</v>
       </c>
       <c r="AM3" s="32">
         <f>Config!$B$6+238</f>
-        <v/>
+        <v>46265.0</v>
       </c>
       <c r="AN3" s="32">
         <f>Config!$B$6+245</f>
-        <v/>
+        <v>46272.0</v>
       </c>
       <c r="AO3" s="32">
         <f>Config!$B$6+252</f>
-        <v/>
+        <v>46279.0</v>
       </c>
       <c r="AP3" s="32">
         <f>Config!$B$6+259</f>
-        <v/>
+        <v>46286.0</v>
       </c>
       <c r="AQ3" s="32">
         <f>Config!$B$6+266</f>
-        <v/>
+        <v>46293.0</v>
       </c>
       <c r="AR3" s="32">
         <f>Config!$B$6+273</f>
-        <v/>
+        <v>46300.0</v>
       </c>
       <c r="AS3" s="32">
         <f>Config!$B$6+280</f>
-        <v/>
+        <v>46307.0</v>
       </c>
       <c r="AT3" s="32">
         <f>Config!$B$6+287</f>
-        <v/>
+        <v>46314.0</v>
       </c>
       <c r="AU3" s="32">
         <f>Config!$B$6+294</f>
-        <v/>
+        <v>46321.0</v>
       </c>
       <c r="AV3" s="32">
         <f>Config!$B$6+301</f>
-        <v/>
+        <v>46328.0</v>
       </c>
       <c r="AW3" s="32">
         <f>Config!$B$6+308</f>
-        <v/>
+        <v>46335.0</v>
       </c>
       <c r="AX3" s="32">
         <f>Config!$B$6+315</f>
-        <v/>
+        <v>46342.0</v>
       </c>
       <c r="AY3" s="32">
         <f>Config!$B$6+322</f>
-        <v/>
+        <v>46349.0</v>
       </c>
       <c r="AZ3" s="32">
         <f>Config!$B$6+329</f>
-        <v/>
+        <v>46356.0</v>
       </c>
       <c r="BA3" s="32">
         <f>Config!$B$6+336</f>
-        <v/>
+        <v>46363.0</v>
       </c>
       <c r="BB3" s="32">
         <f>Config!$B$6+343</f>
-        <v/>
+        <v>46370.0</v>
       </c>
       <c r="BC3" s="32">
         <f>Config!$B$6+350</f>
-        <v/>
+        <v>46377.0</v>
       </c>
       <c r="BD3" s="32">
         <f>Config!$B$6+357</f>
-        <v/>
+        <v>46384.0</v>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
@@ -5115,211 +5122,211 @@
       </c>
       <c r="E30" s="35">
         <f>COUNTIF(E5:E28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F30" s="35">
         <f>COUNTIF(F5:F28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G30" s="35">
         <f>COUNTIF(G5:G28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H30" s="35">
         <f>COUNTIF(H5:H28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I30" s="35">
         <f>COUNTIF(I5:I28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J30" s="35">
         <f>COUNTIF(J5:J28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K30" s="35">
         <f>COUNTIF(K5:K28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L30" s="35">
         <f>COUNTIF(L5:L28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="M30" s="35">
         <f>COUNTIF(M5:M28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N30" s="35">
         <f>COUNTIF(N5:N28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O30" s="35">
         <f>COUNTIF(O5:O28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P30" s="35">
         <f>COUNTIF(P5:P28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q30" s="35">
         <f>COUNTIF(Q5:Q28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="R30" s="35">
         <f>COUNTIF(R5:R28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S30" s="35">
         <f>COUNTIF(S5:S28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="T30" s="35">
         <f>COUNTIF(T5:T28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="U30" s="35">
         <f>COUNTIF(U5:U28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="V30" s="35">
         <f>COUNTIF(V5:V28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="W30" s="35">
         <f>COUNTIF(W5:W28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="X30" s="35">
         <f>COUNTIF(X5:X28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Y30" s="35">
         <f>COUNTIF(Y5:Y28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Z30" s="35">
         <f>COUNTIF(Z5:Z28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AA30" s="35">
         <f>COUNTIF(AA5:AA28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AB30" s="35">
         <f>COUNTIF(AB5:AB28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC30" s="35">
         <f>COUNTIF(AC5:AC28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AD30" s="35">
         <f>COUNTIF(AD5:AD28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AE30" s="35">
         <f>COUNTIF(AE5:AE28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AF30" s="35">
         <f>COUNTIF(AF5:AF28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AG30" s="35">
         <f>COUNTIF(AG5:AG28,"Sim")</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="AH30" s="35">
         <f>COUNTIF(AH5:AH28,"Sim")</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="AI30" s="35">
         <f>COUNTIF(AI5:AI28,"Sim")</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="AJ30" s="35">
         <f>COUNTIF(AJ5:AJ28,"Sim")</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="AK30" s="35">
         <f>COUNTIF(AK5:AK28,"Sim")</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AL30" s="35">
         <f>COUNTIF(AL5:AL28,"Sim")</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="AM30" s="35">
         <f>COUNTIF(AM5:AM28,"Sim")</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="AN30" s="35">
         <f>COUNTIF(AN5:AN28,"Sim")</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="AO30" s="35">
         <f>COUNTIF(AO5:AO28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AP30" s="35">
         <f>COUNTIF(AP5:AP28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AQ30" s="35">
         <f>COUNTIF(AQ5:AQ28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AR30" s="35">
         <f>COUNTIF(AR5:AR28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AS30" s="35">
         <f>COUNTIF(AS5:AS28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AT30" s="35">
         <f>COUNTIF(AT5:AT28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AU30" s="35">
         <f>COUNTIF(AU5:AU28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AV30" s="35">
         <f>COUNTIF(AV5:AV28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AW30" s="35">
         <f>COUNTIF(AW5:AW28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AX30" s="35">
         <f>COUNTIF(AX5:AX28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AY30" s="35">
         <f>COUNTIF(AY5:AY28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AZ30" s="35">
         <f>COUNTIF(AZ5:AZ28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="BA30" s="35">
         <f>COUNTIF(BA5:BA28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="BB30" s="35">
         <f>COUNTIF(BB5:BB28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="BC30" s="35">
         <f>COUNTIF(BC5:BC28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="BD30" s="35">
         <f>COUNTIF(BD5:BD28,"Sim")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -5330,211 +5337,211 @@
       </c>
       <c r="E31" s="35">
         <f>COUNTIF(E5:E28,"Sim")+COUNTIF(E5:E28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F31" s="35">
         <f>COUNTIF(F5:F28,"Sim")+COUNTIF(F5:F28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G31" s="35">
         <f>COUNTIF(G5:G28,"Sim")+COUNTIF(G5:G28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H31" s="35">
         <f>COUNTIF(H5:H28,"Sim")+COUNTIF(H5:H28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I31" s="35">
         <f>COUNTIF(I5:I28,"Sim")+COUNTIF(I5:I28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J31" s="35">
         <f>COUNTIF(J5:J28,"Sim")+COUNTIF(J5:J28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K31" s="35">
         <f>COUNTIF(K5:K28,"Sim")+COUNTIF(K5:K28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L31" s="35">
         <f>COUNTIF(L5:L28,"Sim")+COUNTIF(L5:L28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="M31" s="35">
         <f>COUNTIF(M5:M28,"Sim")+COUNTIF(M5:M28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N31" s="35">
         <f>COUNTIF(N5:N28,"Sim")+COUNTIF(N5:N28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O31" s="35">
         <f>COUNTIF(O5:O28,"Sim")+COUNTIF(O5:O28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P31" s="35">
         <f>COUNTIF(P5:P28,"Sim")+COUNTIF(P5:P28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q31" s="35">
         <f>COUNTIF(Q5:Q28,"Sim")+COUNTIF(Q5:Q28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="R31" s="35">
         <f>COUNTIF(R5:R28,"Sim")+COUNTIF(R5:R28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S31" s="35">
         <f>COUNTIF(S5:S28,"Sim")+COUNTIF(S5:S28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="T31" s="35">
         <f>COUNTIF(T5:T28,"Sim")+COUNTIF(T5:T28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="U31" s="35">
         <f>COUNTIF(U5:U28,"Sim")+COUNTIF(U5:U28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="V31" s="35">
         <f>COUNTIF(V5:V28,"Sim")+COUNTIF(V5:V28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="W31" s="35">
         <f>COUNTIF(W5:W28,"Sim")+COUNTIF(W5:W28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="X31" s="35">
         <f>COUNTIF(X5:X28,"Sim")+COUNTIF(X5:X28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Y31" s="35">
         <f>COUNTIF(Y5:Y28,"Sim")+COUNTIF(Y5:Y28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Z31" s="35">
         <f>COUNTIF(Z5:Z28,"Sim")+COUNTIF(Z5:Z28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AA31" s="35">
         <f>COUNTIF(AA5:AA28,"Sim")+COUNTIF(AA5:AA28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AB31" s="35">
         <f>COUNTIF(AB5:AB28,"Sim")+COUNTIF(AB5:AB28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC31" s="35">
         <f>COUNTIF(AC5:AC28,"Sim")+COUNTIF(AC5:AC28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AD31" s="35">
         <f>COUNTIF(AD5:AD28,"Sim")+COUNTIF(AD5:AD28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AE31" s="35">
         <f>COUNTIF(AE5:AE28,"Sim")+COUNTIF(AE5:AE28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AF31" s="35">
         <f>COUNTIF(AF5:AF28,"Sim")+COUNTIF(AF5:AF28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AG31" s="35">
         <f>COUNTIF(AG5:AG28,"Sim")+COUNTIF(AG5:AG28,"Não")</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AH31" s="35">
         <f>COUNTIF(AH5:AH28,"Sim")+COUNTIF(AH5:AH28,"Não")</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AI31" s="35">
         <f>COUNTIF(AI5:AI28,"Sim")+COUNTIF(AI5:AI28,"Não")</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AJ31" s="35">
         <f>COUNTIF(AJ5:AJ28,"Sim")+COUNTIF(AJ5:AJ28,"Não")</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AK31" s="35">
         <f>COUNTIF(AK5:AK28,"Sim")+COUNTIF(AK5:AK28,"Não")</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AL31" s="35">
         <f>COUNTIF(AL5:AL28,"Sim")+COUNTIF(AL5:AL28,"Não")</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AM31" s="35">
         <f>COUNTIF(AM5:AM28,"Sim")+COUNTIF(AM5:AM28,"Não")</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AN31" s="35">
         <f>COUNTIF(AN5:AN28,"Sim")+COUNTIF(AN5:AN28,"Não")</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AO31" s="35">
         <f>COUNTIF(AO5:AO28,"Sim")+COUNTIF(AO5:AO28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AP31" s="35">
         <f>COUNTIF(AP5:AP28,"Sim")+COUNTIF(AP5:AP28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AQ31" s="35">
         <f>COUNTIF(AQ5:AQ28,"Sim")+COUNTIF(AQ5:AQ28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AR31" s="35">
         <f>COUNTIF(AR5:AR28,"Sim")+COUNTIF(AR5:AR28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AS31" s="35">
         <f>COUNTIF(AS5:AS28,"Sim")+COUNTIF(AS5:AS28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AT31" s="35">
         <f>COUNTIF(AT5:AT28,"Sim")+COUNTIF(AT5:AT28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AU31" s="35">
         <f>COUNTIF(AU5:AU28,"Sim")+COUNTIF(AU5:AU28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AV31" s="35">
         <f>COUNTIF(AV5:AV28,"Sim")+COUNTIF(AV5:AV28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AW31" s="35">
         <f>COUNTIF(AW5:AW28,"Sim")+COUNTIF(AW5:AW28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AX31" s="35">
         <f>COUNTIF(AX5:AX28,"Sim")+COUNTIF(AX5:AX28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AY31" s="35">
         <f>COUNTIF(AY5:AY28,"Sim")+COUNTIF(AY5:AY28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AZ31" s="35">
         <f>COUNTIF(AZ5:AZ28,"Sim")+COUNTIF(AZ5:AZ28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="BA31" s="35">
         <f>COUNTIF(BA5:BA28,"Sim")+COUNTIF(BA5:BA28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="BB31" s="35">
         <f>COUNTIF(BB5:BB28,"Sim")+COUNTIF(BB5:BB28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="BC31" s="35">
         <f>COUNTIF(BC5:BC28,"Sim")+COUNTIF(BC5:BC28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="BD31" s="35">
         <f>COUNTIF(BD5:BD28,"Sim")+COUNTIF(BD5:BD28,"Não")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -5545,211 +5552,211 @@
       </c>
       <c r="E32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="F32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="G32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="H32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="I32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="J32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="K32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="L32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="M32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="N32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="O32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="P32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="Q32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="R32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="S32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="T32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="U32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="V32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="W32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="X32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="Y32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="Z32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AA32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AB32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AC32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AD32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AE32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AF32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AG32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AH32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AI32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AJ32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AK32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AL32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AM32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AN32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AO32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AP32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AQ32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AR32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AS32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AT32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AU32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AV32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AW32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AX32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AY32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="AZ32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="BA32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="BB32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="BC32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="BD32" s="35">
         <f>COUNTA($B$5:$B$28)</f>
-        <v/>
+        <v>9</v>
       </c>
     </row>
     <row r="33">
@@ -5872,35 +5879,35 @@
       </c>
       <c r="AG33" s="23">
         <f>IF(AG31=0,"",AG30/AG32)</f>
-        <v/>
+        <v>0.666666666666667</v>
       </c>
       <c r="AH33" s="23">
         <f>IF(AH31=0,"",AH30/AH32)</f>
-        <v/>
+        <v>0.777777777777778</v>
       </c>
       <c r="AI33" s="23">
         <f>IF(AI31=0,"",AI30/AI32)</f>
-        <v/>
+        <v>0.888888888888889</v>
       </c>
       <c r="AJ33" s="23">
         <f>IF(AJ31=0,"",AJ30/AJ32)</f>
-        <v/>
+        <v>0.888888888888889</v>
       </c>
       <c r="AK33" s="23">
         <f>IF(AK31=0,"",AK30/AK32)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="AL33" s="23">
         <f>IF(AL31=0,"",AL30/AL32)</f>
-        <v/>
+        <v>0.777777777777778</v>
       </c>
       <c r="AM33" s="23">
         <f>IF(AM31=0,"",AM30/AM32)</f>
-        <v/>
+        <v>0.777777777777778</v>
       </c>
       <c r="AN33" s="23">
         <f>IF(AN31=0,"",AN30/AN32)</f>
-        <v/>
+        <v>0.777777777777778</v>
       </c>
       <c r="AO33" s="23">
         <f>IF(AO31=0,"",AO30/AO32)</f>
@@ -5975,211 +5982,211 @@
       </c>
       <c r="E34" s="35">
         <f>SUMIF(E5:E28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F34" s="35">
         <f>SUMIF(F5:F28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G34" s="35">
         <f>SUMIF(G5:G28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H34" s="35">
         <f>SUMIF(H5:H28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I34" s="35">
         <f>SUMIF(I5:I28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J34" s="35">
         <f>SUMIF(J5:J28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K34" s="35">
         <f>SUMIF(K5:K28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L34" s="35">
         <f>SUMIF(L5:L28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="M34" s="35">
         <f>SUMIF(M5:M28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N34" s="35">
         <f>SUMIF(N5:N28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O34" s="35">
         <f>SUMIF(O5:O28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P34" s="35">
         <f>SUMIF(P5:P28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q34" s="35">
         <f>SUMIF(Q5:Q28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="R34" s="35">
         <f>SUMIF(R5:R28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S34" s="35">
         <f>SUMIF(S5:S28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="T34" s="35">
         <f>SUMIF(T5:T28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="U34" s="35">
         <f>SUMIF(U5:U28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="V34" s="35">
         <f>SUMIF(V5:V28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="W34" s="35">
         <f>SUMIF(W5:W28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="X34" s="35">
         <f>SUMIF(X5:X28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Y34" s="35">
         <f>SUMIF(Y5:Y28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Z34" s="35">
         <f>SUMIF(Z5:Z28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AA34" s="35">
         <f>SUMIF(AA5:AA28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AB34" s="35">
         <f>SUMIF(AB5:AB28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC34" s="35">
         <f>SUMIF(AC5:AC28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AD34" s="35">
         <f>SUMIF(AD5:AD28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AE34" s="35">
         <f>SUMIF(AE5:AE28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AF34" s="35">
         <f>SUMIF(AF5:AF28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AG34" s="35">
         <f>SUMIF(AG5:AG28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>19</v>
       </c>
       <c r="AH34" s="35">
         <f>SUMIF(AH5:AH28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>24</v>
       </c>
       <c r="AI34" s="35">
         <f>SUMIF(AI5:AI28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>27</v>
       </c>
       <c r="AJ34" s="35">
         <f>SUMIF(AJ5:AJ28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>27</v>
       </c>
       <c r="AK34" s="35">
         <f>SUMIF(AK5:AK28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>30</v>
       </c>
       <c r="AL34" s="35">
         <f>SUMIF(AL5:AL28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>23</v>
       </c>
       <c r="AM34" s="35">
         <f>SUMIF(AM5:AM28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>24</v>
       </c>
       <c r="AN34" s="35">
         <f>SUMIF(AN5:AN28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>25</v>
       </c>
       <c r="AO34" s="35">
         <f>SUMIF(AO5:AO28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AP34" s="35">
         <f>SUMIF(AP5:AP28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AQ34" s="35">
         <f>SUMIF(AQ5:AQ28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AR34" s="35">
         <f>SUMIF(AR5:AR28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AS34" s="35">
         <f>SUMIF(AS5:AS28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AT34" s="35">
         <f>SUMIF(AT5:AT28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AU34" s="35">
         <f>SUMIF(AU5:AU28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AV34" s="35">
         <f>SUMIF(AV5:AV28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AW34" s="35">
         <f>SUMIF(AW5:AW28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AX34" s="35">
         <f>SUMIF(AX5:AX28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AY34" s="35">
         <f>SUMIF(AY5:AY28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AZ34" s="35">
         <f>SUMIF(AZ5:AZ28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="BA34" s="35">
         <f>SUMIF(BA5:BA28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="BB34" s="35">
         <f>SUMIF(BB5:BB28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="BC34" s="35">
         <f>SUMIF(BC5:BC28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="BD34" s="35">
         <f>SUMIF(BD5:BD28,"Sim",$C$5:$C$28)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="35">

</xml_diff>